<commit_message>
First run with self-learning agent. Execution of WBS 0.4 rev_Grant.
</commit_message>
<xml_diff>
--- a/docs/Import/Application Data Export.xlsx
+++ b/docs/Import/Application Data Export.xlsx
@@ -1563,9 +1563,9 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101006FC0B6920867EF44858ED15B3E78E281" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dd529591f4304f7813924d611895613d">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="8affeb01-2cc2-4424-8643-f03aa7b6b403" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e4efdb5393fd44f5979c82165f4d0946" ns2:_="">
-    <xsd:import namespace="8affeb01-2cc2-4424-8643-f03aa7b6b403"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bfcf18f7e381c9b6f73f745d0af776b2">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9a072e1abc47c2a4da4cb59bf3931f34" ns2:_="">
+    <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1582,7 +1582,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="8affeb01-2cc2-4424-8643-f03aa7b6b403" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="f28f5036-0c97-4fb2-9995-e6511ad4535b" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -1716,7 +1716,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14FC01CE-D660-4EBE-9B8F-CE933FB05C08}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9196091E-4677-4EF5-A1A6-1E7D4A865B9B}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Docusign Workflows are delivered and verified. Ready for testing.
</commit_message>
<xml_diff>
--- a/docs/Import/Application Data Export.xlsx
+++ b/docs/Import/Application Data Export.xlsx
@@ -1563,9 +1563,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bfcf18f7e381c9b6f73f745d0af776b2">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9a072e1abc47c2a4da4cb59bf3931f34" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010019BFD6B84F7029419816FFCF5AF812DE" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae75f7d6110eb3c01e30b5864ecce8d9">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f28f5036-0c97-4fb2-9995-e6511ad4535b" xmlns:ns3="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5f758225586994ab2ed7147b7dc97d7e" ns2:_="" ns3:_="">
     <xsd:import namespace="f28f5036-0c97-4fb2-9995-e6511ad4535b"/>
+    <xsd:import namespace="d3a2e4d4-5189-48ac-a210-e1294fbd99f3"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -1575,6 +1576,11 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -1599,6 +1605,43 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="3edfda32-ed56-4dd9-bd64-14fdcb8b12da" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{309b44fd-1af0-4c99-971b-3abc3e199a55}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="d3a2e4d4-5189-48ac-a210-e1294fbd99f3">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -1711,12 +1754,17 @@
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="f28f5036-0c97-4fb2-9995-e6511ad4535b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d3a2e4d4-5189-48ac-a210-e1294fbd99f3" xsi:nil="true"/>
+  </documentManagement>
 </p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9196091E-4677-4EF5-A1A6-1E7D4A865B9B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6C91D161-351B-49A4-ADFF-1860FF7EE3BA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>